<commit_message>
Change frontend to reflect the endpoints, add data enrichment component allowing the user to fill in information missing from the csv
</commit_message>
<xml_diff>
--- a/csvTest.xlsx
+++ b/csvTest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timco\Desktop\SoftwareProject\gosmartlib\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7948348-7451-4333-8BF6-9FBD9523EE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92732A40-457A-4FD3-8209-DBD783B06E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6525" yWindow="990" windowWidth="26070" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6870" yWindow="1335" windowWidth="26070" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Faulty" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Remove taal/beschrijving metadata from the csv fields, add conflicting isbn decision check, prevent backend google books api rate limiting
</commit_message>
<xml_diff>
--- a/csvTest.xlsx
+++ b/csvTest.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timco\Desktop\SoftwareProject\gosmartlib\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92732A40-457A-4FD3-8209-DBD783B06E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BEB15D-B1D3-41E3-B6A7-6E56A39B7A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6870" yWindow="1335" windowWidth="26070" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6870" yWindow="1335" windowWidth="26070" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Faulty" sheetId="2" r:id="rId1"/>
     <sheet name="Working" sheetId="3" r:id="rId2"/>
-    <sheet name="Conflict-todo" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="20">
   <si>
     <t>Titel</t>
   </si>
@@ -56,12 +55,6 @@
     <t>Campus</t>
   </si>
   <si>
-    <t>Taal</t>
-  </si>
-  <si>
-    <t>Beschrijving</t>
-  </si>
-  <si>
     <t>De Bron</t>
   </si>
   <si>
@@ -71,9 +64,6 @@
     <t>Campus Z</t>
   </si>
   <si>
-    <t>NEDERLANDS</t>
-  </si>
-  <si>
     <t>De lotus en de waringinboom</t>
   </si>
   <si>
@@ -89,9 +79,6 @@
     <t>Philip Pullman</t>
   </si>
   <si>
-    <t>ENGELS</t>
-  </si>
-  <si>
     <t>Campus A</t>
   </si>
   <si>
@@ -99,9 +86,6 @@
   </si>
   <si>
     <t>Alaa</t>
-  </si>
-  <si>
-    <t>Conflicting info between existing Item &lt;-&gt; user input fields from csv</t>
   </si>
 </sst>
 </file>
@@ -131,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -178,45 +162,17 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,23 +453,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C87E3B4-7637-4234-8AE5-66605123FBD4}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.28515625" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5703125" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -541,69 +495,54 @@
       <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>9789047716808</v>
       </c>
       <c r="D2">
         <v>4</v>
       </c>
       <c r="I2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="6">
+      <c r="C3" s="5">
         <v>97890477185740</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
-      <c r="J3" t="s">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>9789044862188</v>
       </c>
-      <c r="J4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="6">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5">
         <v>9780241458709</v>
       </c>
       <c r="D5">
@@ -615,39 +554,29 @@
       <c r="F5">
         <v>2</v>
       </c>
-      <c r="J5" t="s">
-        <v>20</v>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1:J1048576" xr:uid="{2C99130C-1C34-4DE3-A702-DE4AFC6258DA}">
-      <formula1>"NEDERLANDS,FRANS,ENGELS,DUITS,ANDERE"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D0160F2-8993-41CA-B972-41645C7BC3B6}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.28515625" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5703125" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -675,21 +604,15 @@
       <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>9789047716808</v>
       </c>
       <c r="D2">
@@ -699,20 +622,17 @@
         <v>4</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="6">
+        <v>13</v>
+      </c>
+      <c r="C3" s="5">
         <v>9789047718574</v>
       </c>
       <c r="D3">
@@ -725,37 +645,31 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>9789044862188</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="6">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5">
         <v>9780241458709</v>
       </c>
       <c r="D5">
@@ -768,87 +682,10 @@
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1:J1048576" xr:uid="{A110DDCA-7098-4917-AA5C-819A55436F88}">
-      <formula1>"NEDERLANDS,FRANS,ENGELS,DUITS,ANDERE"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{514FA362-CE0F-4AAA-8756-F99FC242E43F}">
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="16.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1:J1048576" xr:uid="{67084ABA-B11B-48B4-9AFE-ADAB3475B6D0}">
-      <formula1>"NEDERLANDS,FRANS,ENGELS,DUITS,ANDERE"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>